<commit_message>
feat: add weapon classes and composable combat skills
</commit_message>
<xml_diff>
--- a/config/excel/CfgCombatFeedback.xlsx
+++ b/config/excel/CfgCombatFeedback.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="48">
   <si>
     <t>ID</t>
   </si>
@@ -143,6 +143,18 @@
   </si>
   <si>
     <t>流血</t>
+  </si>
+  <si>
+    <t>orbit_status</t>
+  </si>
+  <si>
+    <t>环身剑阵</t>
+  </si>
+  <si>
+    <t>regeneration_status</t>
+  </si>
+  <si>
+    <t>复苏</t>
   </si>
 </sst>
 </file>
@@ -519,7 +531,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="4" width="20" customWidth="1"/>
@@ -759,7 +771,7 @@
         <v>1</v>
       </c>
       <c r="C8">
-        <v>1001</v>
+        <v>5</v>
       </c>
       <c r="D8" t="b">
         <v>0</v>
@@ -943,8 +955,72 @@
         <v>0</v>
       </c>
     </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>44</v>
+      </c>
+      <c r="B14">
+        <v>6</v>
+      </c>
+      <c r="C14">
+        <v>100</v>
+      </c>
+      <c r="D14" t="b">
+        <v>0</v>
+      </c>
+      <c r="E14" t="s">
+        <v>45</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14">
+        <v>0.85</v>
+      </c>
+      <c r="H14">
+        <v>0.25</v>
+      </c>
+      <c r="I14" t="b">
+        <v>0</v>
+      </c>
+      <c r="J14" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>46</v>
+      </c>
+      <c r="B15">
+        <v>6</v>
+      </c>
+      <c r="C15">
+        <v>101</v>
+      </c>
+      <c r="D15" t="b">
+        <v>0</v>
+      </c>
+      <c r="E15" t="s">
+        <v>47</v>
+      </c>
+      <c r="F15">
+        <v>0.35</v>
+      </c>
+      <c r="G15">
+        <v>1</v>
+      </c>
+      <c r="H15">
+        <v>0.45</v>
+      </c>
+      <c r="I15" t="b">
+        <v>0</v>
+      </c>
+      <c r="J15" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>